<commit_message>
#4 Client and eSpark BOM Completed with LCD Peripheral
</commit_message>
<xml_diff>
--- a/Design-Files/MVP-Dash-v1.0/BOM/Client_BOM.xlsx
+++ b/Design-Files/MVP-Dash-v1.0/BOM/Client_BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1249" uniqueCount="741">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1256" uniqueCount="746">
   <si>
     <t>#</t>
   </si>
@@ -2242,6 +2242,21 @@
   </si>
   <si>
     <t>Do Not Place</t>
+  </si>
+  <si>
+    <t>Peripherals</t>
+  </si>
+  <si>
+    <t>LCD</t>
+  </si>
+  <si>
+    <t>7.0 inch 280*1424,HDMI Interfac</t>
+  </si>
+  <si>
+    <t>KD050FHFID103</t>
+  </si>
+  <si>
+    <t>SHENZHEN STARTEK ELECTRONIC TECHNOLOGYCO.,LTD</t>
   </si>
 </sst>
 </file>
@@ -2459,9 +2474,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2470,6 +2482,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2758,7 +2773,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K179"/>
+  <dimension ref="A1:K180"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="4" style="4" bestFit="1" customWidth="1"/>
@@ -2782,9 +2797,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -3628,28 +3643,28 @@
       <c r="C28" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="E28" s="16" t="s">
+      <c r="E28" s="15" t="s">
         <v>236</v>
       </c>
-      <c r="F28" s="15" t="s">
+      <c r="F28" s="14" t="s">
         <v>388</v>
       </c>
-      <c r="G28" s="16" t="s">
+      <c r="G28" s="15" t="s">
         <v>477</v>
       </c>
-      <c r="H28" s="15" t="s">
+      <c r="H28" s="14" t="s">
         <v>612</v>
       </c>
-      <c r="I28" s="15" t="s">
+      <c r="I28" s="14" t="s">
         <v>677</v>
       </c>
-      <c r="J28" s="15">
-        <v>1</v>
-      </c>
-      <c r="K28" s="17" t="s">
+      <c r="J28" s="14">
+        <v>1</v>
+      </c>
+      <c r="K28" s="16" t="s">
         <v>740</v>
       </c>
     </row>
@@ -5608,28 +5623,28 @@
       <c r="C90" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D90" s="15" t="s">
+      <c r="D90" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="E90" s="16" t="s">
+      <c r="E90" s="15" t="s">
         <v>296</v>
       </c>
-      <c r="F90" s="15" t="s">
+      <c r="F90" s="14" t="s">
         <v>426</v>
       </c>
-      <c r="G90" s="16" t="s">
+      <c r="G90" s="15" t="s">
         <v>524</v>
       </c>
-      <c r="H90" s="15" t="s">
+      <c r="H90" s="14" t="s">
         <v>613</v>
       </c>
-      <c r="I90" s="15" t="s">
+      <c r="I90" s="14" t="s">
         <v>677</v>
       </c>
-      <c r="J90" s="15">
-        <v>1</v>
-      </c>
-      <c r="K90" s="17" t="s">
+      <c r="J90" s="14">
+        <v>1</v>
+      </c>
+      <c r="K90" s="16" t="s">
         <v>740</v>
       </c>
     </row>
@@ -6378,28 +6393,28 @@
       <c r="C114" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D114" s="15" t="s">
+      <c r="D114" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="E114" s="16" t="s">
+      <c r="E114" s="15" t="s">
         <v>298</v>
       </c>
-      <c r="F114" s="15" t="s">
+      <c r="F114" s="14" t="s">
         <v>425</v>
       </c>
-      <c r="G114" s="16" t="s">
+      <c r="G114" s="15" t="s">
         <v>526</v>
       </c>
-      <c r="H114" s="15" t="s">
+      <c r="H114" s="14" t="s">
         <v>613</v>
       </c>
-      <c r="I114" s="15" t="s">
+      <c r="I114" s="14" t="s">
         <v>677</v>
       </c>
-      <c r="J114" s="15">
-        <v>1</v>
-      </c>
-      <c r="K114" s="17" t="s">
+      <c r="J114" s="14">
+        <v>1</v>
+      </c>
+      <c r="K114" s="16" t="s">
         <v>740</v>
       </c>
     </row>
@@ -6700,28 +6715,28 @@
       <c r="C124" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D124" s="15" t="s">
+      <c r="D124" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="E124" s="16" t="s">
+      <c r="E124" s="15" t="s">
         <v>312</v>
       </c>
-      <c r="F124" s="15" t="s">
+      <c r="F124" s="14" t="s">
         <v>425</v>
       </c>
-      <c r="G124" s="16" t="s">
+      <c r="G124" s="15" t="s">
         <v>540</v>
       </c>
-      <c r="H124" s="15" t="s">
+      <c r="H124" s="14" t="s">
         <v>613</v>
       </c>
-      <c r="I124" s="15" t="s">
+      <c r="I124" s="14" t="s">
         <v>677</v>
       </c>
-      <c r="J124" s="15">
-        <v>1</v>
-      </c>
-      <c r="K124" s="17" t="s">
+      <c r="J124" s="14">
+        <v>1</v>
+      </c>
+      <c r="K124" s="16" t="s">
         <v>740</v>
       </c>
     </row>
@@ -8484,6 +8499,37 @@
         <v>1</v>
       </c>
       <c r="K179" s="7"/>
+    </row>
+    <row r="180" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B180" s="11">
+        <f>ROW(B180) - ROW($B$2)</f>
+        <v>178</v>
+      </c>
+      <c r="C180" s="13" t="s">
+        <v>741</v>
+      </c>
+      <c r="D180" s="7" t="s">
+        <v>742</v>
+      </c>
+      <c r="E180" s="7" t="s">
+        <v>743</v>
+      </c>
+      <c r="F180" s="7" t="s">
+        <v>739</v>
+      </c>
+      <c r="G180" s="7" t="s">
+        <v>744</v>
+      </c>
+      <c r="H180" s="7" t="s">
+        <v>745</v>
+      </c>
+      <c r="I180" s="7" t="s">
+        <v>737</v>
+      </c>
+      <c r="J180" s="7">
+        <v>1</v>
+      </c>
+      <c r="K180" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
#6 Updated Client BOM
</commit_message>
<xml_diff>
--- a/Design-Files/MVP-Dash-v1.0/BOM/Client_BOM.xlsx
+++ b/Design-Files/MVP-Dash-v1.0/BOM/Client_BOM.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="776">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="790">
   <si>
     <t>#</t>
   </si>
@@ -2355,6 +2355,48 @@
   </si>
   <si>
     <t>37.4MHz</t>
+  </si>
+  <si>
+    <t>Peripherals</t>
+  </si>
+  <si>
+    <t>LCD</t>
+  </si>
+  <si>
+    <t>7.0 inch 280*1424,HDMI Interfac</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>KD050FHFID103</t>
+  </si>
+  <si>
+    <t>SHENZHEN STARTEK ELECTRONIC TECHNOLOGYCO.,LTD</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mating Connector </t>
+  </si>
+  <si>
+    <t>3 35P 4mm - Automobile Connectors ROHS</t>
+  </si>
+  <si>
+    <t>K776280H-35-PTW</t>
+  </si>
+  <si>
+    <t>XKB Connection</t>
+  </si>
+  <si>
+    <t>Mating pin Terminal</t>
+  </si>
+  <si>
+    <t>Automobile Connectors ROHS</t>
+  </si>
+  <si>
+    <t>K776280T-PSN</t>
   </si>
 </sst>
 </file>
@@ -2367,7 +2409,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="31">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2433,8 +2475,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2982,28 +3038,19 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -3012,122 +3059,131 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3180,6 +3236,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3507,7 +3572,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K184"/>
+  <dimension ref="A1:K187"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.14285714285714" customWidth="1"/>
@@ -9333,6 +9398,99 @@
       </c>
       <c r="K184" s="12"/>
     </row>
+    <row r="185" ht="36.75" spans="2:11">
+      <c r="B185" s="20">
+        <f>ROW(B185)-ROW($B$2)</f>
+        <v>183</v>
+      </c>
+      <c r="C185" s="21" t="s">
+        <v>776</v>
+      </c>
+      <c r="D185" s="22" t="s">
+        <v>777</v>
+      </c>
+      <c r="E185" s="22" t="s">
+        <v>778</v>
+      </c>
+      <c r="F185" s="22" t="s">
+        <v>779</v>
+      </c>
+      <c r="G185" s="22" t="s">
+        <v>780</v>
+      </c>
+      <c r="H185" s="22" t="s">
+        <v>781</v>
+      </c>
+      <c r="I185" s="22" t="s">
+        <v>782</v>
+      </c>
+      <c r="J185" s="22">
+        <v>1</v>
+      </c>
+      <c r="K185" s="22"/>
+    </row>
+    <row r="186" ht="24.75" spans="2:11">
+      <c r="B186" s="20">
+        <f>ROW(B186)-ROW($B$2)</f>
+        <v>184</v>
+      </c>
+      <c r="C186" s="21" t="s">
+        <v>776</v>
+      </c>
+      <c r="D186" s="22" t="s">
+        <v>783</v>
+      </c>
+      <c r="E186" s="22" t="s">
+        <v>784</v>
+      </c>
+      <c r="F186" s="22" t="s">
+        <v>779</v>
+      </c>
+      <c r="G186" s="22" t="s">
+        <v>785</v>
+      </c>
+      <c r="H186" s="22" t="s">
+        <v>786</v>
+      </c>
+      <c r="I186" s="22" t="s">
+        <v>782</v>
+      </c>
+      <c r="J186" s="22">
+        <v>1</v>
+      </c>
+      <c r="K186" s="22"/>
+    </row>
+    <row r="187" ht="15.75" spans="2:11">
+      <c r="B187" s="20">
+        <f>ROW(B187)-ROW($B$2)</f>
+        <v>185</v>
+      </c>
+      <c r="C187" s="21" t="s">
+        <v>776</v>
+      </c>
+      <c r="D187" s="22" t="s">
+        <v>787</v>
+      </c>
+      <c r="E187" s="22" t="s">
+        <v>788</v>
+      </c>
+      <c r="F187" s="22" t="s">
+        <v>779</v>
+      </c>
+      <c r="G187" s="22" t="s">
+        <v>789</v>
+      </c>
+      <c r="H187" s="22" t="s">
+        <v>786</v>
+      </c>
+      <c r="I187" s="22" t="s">
+        <v>782</v>
+      </c>
+      <c r="J187" s="22">
+        <v>35</v>
+      </c>
+      <c r="K187" s="22"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>

</xml_diff>

<commit_message>
J4 marked DNP #4
</commit_message>
<xml_diff>
--- a/Design-Files/MVP-Dash-v1.0/BOM/Client_BOM.xlsx
+++ b/Design-Files/MVP-Dash-v1.0/BOM/Client_BOM.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\alastair-baronessalpha\Design-Files\MVP-Dash-v1.0\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11850"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11850"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1274" uniqueCount="790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="790">
   <si>
     <t>#</t>
   </si>
@@ -2402,14 +2407,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="31">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2496,151 +2495,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2659,194 +2529,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="16">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -2937,253 +2621,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3226,9 +2668,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3247,68 +2686,36 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="0003A4CB"/>
-      <color rgb="002CD0B2"/>
+      <color rgb="FF03A4CB"/>
+      <color rgb="FF2CD0B2"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -3566,29 +2973,30 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K187"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.14285714285714" customWidth="1"/>
-    <col min="2" max="2" width="5.14285714285714" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" customWidth="1"/>
+    <col min="2" max="2" width="5.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5714285714286" customWidth="1"/>
-    <col min="7" max="7" width="33.4285714285714" customWidth="1"/>
-    <col min="8" max="8" width="21.4285714285714" customWidth="1"/>
-    <col min="9" max="9" width="17.8571428571429" customWidth="1"/>
-    <col min="10" max="10" width="16.7142857142857" customWidth="1"/>
-    <col min="11" max="11" width="29.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:11">
+    <row r="1" spans="1:11">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3597,11 +3005,11 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-    </row>
-    <row r="2" ht="15.75" spans="1:11">
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -3634,7 +3042,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="15.75" spans="1:11">
+    <row r="3" spans="1:11">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
         <f>ROW(B3)-ROW($B$2)</f>
@@ -3666,7 +3074,7 @@
       </c>
       <c r="K3" s="9"/>
     </row>
-    <row r="4" ht="24.75" spans="1:11">
+    <row r="4" spans="1:11" ht="24">
       <c r="A4" s="2"/>
       <c r="B4" s="7">
         <f t="shared" ref="B4:B184" si="0">ROW(B4)-ROW($B$2)</f>
@@ -3698,7 +3106,7 @@
       </c>
       <c r="K4" s="12"/>
     </row>
-    <row r="5" ht="15.75" spans="1:11">
+    <row r="5" spans="1:11">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
         <f>ROW(B5)-ROW($B$2)</f>
@@ -3728,7 +3136,7 @@
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" ht="24.75" spans="1:11">
+    <row r="6" spans="1:11" ht="24">
       <c r="A6" s="2"/>
       <c r="B6" s="7">
         <f t="shared" si="0"/>
@@ -3760,7 +3168,7 @@
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" ht="15.75" spans="1:11">
+    <row r="7" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
         <f>ROW(B7)-ROW($B$2)</f>
@@ -3792,7 +3200,7 @@
       </c>
       <c r="K7" s="9"/>
     </row>
-    <row r="8" ht="36.75" spans="1:11">
+    <row r="8" spans="1:11" ht="36">
       <c r="A8" s="2"/>
       <c r="B8" s="7">
         <f t="shared" si="0"/>
@@ -3824,7 +3232,7 @@
       </c>
       <c r="K8" s="12"/>
     </row>
-    <row r="9" ht="15.75" spans="1:11">
+    <row r="9" spans="1:11">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
         <f>ROW(B9)-ROW($B$2)</f>
@@ -3854,7 +3262,7 @@
       </c>
       <c r="K9" s="9"/>
     </row>
-    <row r="10" ht="15.75" spans="1:11">
+    <row r="10" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
         <f t="shared" si="0"/>
@@ -3886,7 +3294,7 @@
       </c>
       <c r="K10" s="12"/>
     </row>
-    <row r="11" ht="15.75" spans="1:11">
+    <row r="11" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
         <f>ROW(B11)-ROW($B$2)</f>
@@ -3918,7 +3326,7 @@
       </c>
       <c r="K11" s="9"/>
     </row>
-    <row r="12" ht="15.75" spans="1:11">
+    <row r="12" spans="1:11">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
         <f t="shared" si="0"/>
@@ -3950,7 +3358,7 @@
       </c>
       <c r="K12" s="12"/>
     </row>
-    <row r="13" ht="15.75" spans="1:11">
+    <row r="13" spans="1:11">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
         <f>ROW(B13)-ROW($B$2)</f>
@@ -3982,7 +3390,7 @@
       </c>
       <c r="K13" s="9"/>
     </row>
-    <row r="14" ht="24.75" spans="1:11">
+    <row r="14" spans="1:11" ht="24">
       <c r="A14" s="2"/>
       <c r="B14" s="7">
         <f t="shared" si="0"/>
@@ -4014,7 +3422,7 @@
       </c>
       <c r="K14" s="12"/>
     </row>
-    <row r="15" ht="108.75" spans="1:11">
+    <row r="15" spans="1:11" ht="108">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
         <f>ROW(B15)-ROW($B$2)</f>
@@ -4046,7 +3454,7 @@
       </c>
       <c r="K15" s="9"/>
     </row>
-    <row r="16" ht="36.75" spans="1:11">
+    <row r="16" spans="1:11" ht="36">
       <c r="A16" s="2"/>
       <c r="B16" s="7">
         <f t="shared" si="0"/>
@@ -4076,7 +3484,7 @@
       </c>
       <c r="K16" s="12"/>
     </row>
-    <row r="17" ht="15.75" spans="1:11">
+    <row r="17" spans="1:11">
       <c r="A17" s="2"/>
       <c r="B17" s="7">
         <f>ROW(B17)-ROW($B$2)</f>
@@ -4108,7 +3516,7 @@
       </c>
       <c r="K17" s="9"/>
     </row>
-    <row r="18" ht="15.75" spans="1:11">
+    <row r="18" spans="1:11">
       <c r="A18" s="2"/>
       <c r="B18" s="7">
         <f t="shared" si="0"/>
@@ -4138,7 +3546,7 @@
       </c>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" ht="60.75" spans="1:11">
+    <row r="19" spans="1:11" ht="60">
       <c r="A19" s="2"/>
       <c r="B19" s="7">
         <f>ROW(B19)-ROW($B$2)</f>
@@ -4170,7 +3578,7 @@
       </c>
       <c r="K19" s="9"/>
     </row>
-    <row r="20" ht="15.75" spans="1:11">
+    <row r="20" spans="1:11">
       <c r="A20" s="2"/>
       <c r="B20" s="7">
         <f t="shared" si="0"/>
@@ -4202,7 +3610,7 @@
       </c>
       <c r="K20" s="12"/>
     </row>
-    <row r="21" ht="24.75" spans="1:11">
+    <row r="21" spans="1:11" ht="24">
       <c r="A21" s="2"/>
       <c r="B21" s="7">
         <f>ROW(B21)-ROW($B$2)</f>
@@ -4234,7 +3642,7 @@
       </c>
       <c r="K21" s="9"/>
     </row>
-    <row r="22" ht="84.75" spans="1:11">
+    <row r="22" spans="1:11" ht="84">
       <c r="A22" s="2"/>
       <c r="B22" s="7">
         <f t="shared" si="0"/>
@@ -4264,7 +3672,7 @@
       </c>
       <c r="K22" s="12"/>
     </row>
-    <row r="23" ht="15.75" spans="1:11">
+    <row r="23" spans="1:11">
       <c r="A23" s="2"/>
       <c r="B23" s="7">
         <f>ROW(B23)-ROW($B$2)</f>
@@ -4296,7 +3704,7 @@
       </c>
       <c r="K23" s="9"/>
     </row>
-    <row r="24" ht="24.75" spans="1:11">
+    <row r="24" spans="1:11" ht="24">
       <c r="A24" s="2"/>
       <c r="B24" s="7">
         <f t="shared" si="0"/>
@@ -4328,7 +3736,7 @@
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" ht="15.75" spans="1:11">
+    <row r="25" spans="1:11">
       <c r="A25" s="2"/>
       <c r="B25" s="7">
         <f>ROW(B25)-ROW($B$2)</f>
@@ -4360,7 +3768,7 @@
       </c>
       <c r="K25" s="9"/>
     </row>
-    <row r="26" ht="36.75" spans="1:11">
+    <row r="26" spans="1:11" ht="36">
       <c r="A26" s="2"/>
       <c r="B26" s="7">
         <f t="shared" si="0"/>
@@ -4392,7 +3800,7 @@
       </c>
       <c r="K26" s="12"/>
     </row>
-    <row r="27" ht="15.75" spans="1:11">
+    <row r="27" spans="1:11">
       <c r="A27" s="2"/>
       <c r="B27" s="7">
         <f>ROW(B27)-ROW($B$2)</f>
@@ -4424,7 +3832,7 @@
       </c>
       <c r="K27" s="9"/>
     </row>
-    <row r="28" ht="15.75" spans="1:11">
+    <row r="28" spans="1:11">
       <c r="A28" s="2"/>
       <c r="B28" s="7">
         <f t="shared" si="0"/>
@@ -4454,11 +3862,11 @@
       <c r="J28" s="14">
         <v>1</v>
       </c>
-      <c r="K28" s="17" t="s">
+      <c r="K28" s="16" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="29" ht="15.75" spans="1:11">
+    <row r="29" spans="1:11">
       <c r="A29" s="2"/>
       <c r="B29" s="7">
         <f>ROW(B29)-ROW($B$2)</f>
@@ -4490,7 +3898,7 @@
       </c>
       <c r="K29" s="9"/>
     </row>
-    <row r="30" ht="15.75" spans="1:11">
+    <row r="30" spans="1:11">
       <c r="A30" s="2"/>
       <c r="B30" s="7">
         <f t="shared" si="0"/>
@@ -4522,7 +3930,7 @@
       </c>
       <c r="K30" s="12"/>
     </row>
-    <row r="31" ht="15.75" spans="1:11">
+    <row r="31" spans="1:11">
       <c r="A31" s="2"/>
       <c r="B31" s="7">
         <f>ROW(B31)-ROW($B$2)</f>
@@ -4554,7 +3962,7 @@
       </c>
       <c r="K31" s="9"/>
     </row>
-    <row r="32" ht="15.75" spans="1:11">
+    <row r="32" spans="1:11">
       <c r="A32" s="2"/>
       <c r="B32" s="7">
         <f t="shared" si="0"/>
@@ -4584,7 +3992,7 @@
       </c>
       <c r="K32" s="12"/>
     </row>
-    <row r="33" ht="15.75" spans="1:11">
+    <row r="33" spans="1:11">
       <c r="A33" s="2"/>
       <c r="B33" s="7">
         <f>ROW(B33)-ROW($B$2)</f>
@@ -4616,7 +4024,7 @@
       </c>
       <c r="K33" s="9"/>
     </row>
-    <row r="34" ht="15.75" spans="1:11">
+    <row r="34" spans="1:11">
       <c r="A34" s="2"/>
       <c r="B34" s="7">
         <f t="shared" si="0"/>
@@ -4646,7 +4054,7 @@
       </c>
       <c r="K34" s="12"/>
     </row>
-    <row r="35" ht="15.75" spans="1:11">
+    <row r="35" spans="1:11">
       <c r="A35" s="2"/>
       <c r="B35" s="7">
         <f>ROW(B35)-ROW($B$2)</f>
@@ -4678,7 +4086,7 @@
       </c>
       <c r="K35" s="9"/>
     </row>
-    <row r="36" ht="36.75" spans="1:11">
+    <row r="36" spans="1:11" ht="36">
       <c r="A36" s="2"/>
       <c r="B36" s="7">
         <f t="shared" si="0"/>
@@ -4708,7 +4116,7 @@
       </c>
       <c r="K36" s="12"/>
     </row>
-    <row r="37" ht="15.75" spans="1:11">
+    <row r="37" spans="1:11">
       <c r="A37" s="2"/>
       <c r="B37" s="7">
         <f>ROW(B37)-ROW($B$2)</f>
@@ -4740,7 +4148,7 @@
       </c>
       <c r="K37" s="9"/>
     </row>
-    <row r="38" ht="15.75" spans="1:11">
+    <row r="38" spans="1:11">
       <c r="A38" s="2"/>
       <c r="B38" s="7">
         <f t="shared" si="0"/>
@@ -4772,7 +4180,7 @@
       </c>
       <c r="K38" s="12"/>
     </row>
-    <row r="39" ht="15.75" spans="1:11">
+    <row r="39" spans="1:11">
       <c r="A39" s="2"/>
       <c r="B39" s="7">
         <f>ROW(B39)-ROW($B$2)</f>
@@ -4804,7 +4212,7 @@
       </c>
       <c r="K39" s="9"/>
     </row>
-    <row r="40" ht="15.75" spans="1:11">
+    <row r="40" spans="1:11">
       <c r="A40" s="2"/>
       <c r="B40" s="7">
         <f t="shared" si="0"/>
@@ -4836,7 +4244,7 @@
       </c>
       <c r="K40" s="12"/>
     </row>
-    <row r="41" ht="15.75" spans="1:11">
+    <row r="41" spans="1:11">
       <c r="A41" s="2"/>
       <c r="B41" s="7">
         <f>ROW(B41)-ROW($B$2)</f>
@@ -4866,7 +4274,7 @@
       </c>
       <c r="K41" s="9"/>
     </row>
-    <row r="42" ht="15.75" spans="1:11">
+    <row r="42" spans="1:11">
       <c r="A42" s="2"/>
       <c r="B42" s="7">
         <f t="shared" si="0"/>
@@ -4896,7 +4304,7 @@
       </c>
       <c r="K42" s="12"/>
     </row>
-    <row r="43" ht="15.75" spans="1:11">
+    <row r="43" spans="1:11">
       <c r="A43" s="2"/>
       <c r="B43" s="7">
         <f>ROW(B43)-ROW($B$2)</f>
@@ -4928,7 +4336,7 @@
       </c>
       <c r="K43" s="9"/>
     </row>
-    <row r="44" ht="15.75" spans="1:11">
+    <row r="44" spans="1:11">
       <c r="A44" s="2"/>
       <c r="B44" s="7">
         <f t="shared" si="0"/>
@@ -4960,7 +4368,7 @@
       </c>
       <c r="K44" s="12"/>
     </row>
-    <row r="45" ht="36.75" spans="1:11">
+    <row r="45" spans="1:11" ht="36">
       <c r="A45" s="2"/>
       <c r="B45" s="7">
         <f>ROW(B45)-ROW($B$2)</f>
@@ -4992,7 +4400,7 @@
       </c>
       <c r="K45" s="9"/>
     </row>
-    <row r="46" ht="24.75" spans="1:11">
+    <row r="46" spans="1:11" ht="24">
       <c r="A46" s="2"/>
       <c r="B46" s="7">
         <f t="shared" si="0"/>
@@ -5022,7 +4430,7 @@
       </c>
       <c r="K46" s="12"/>
     </row>
-    <row r="47" ht="36.75" spans="1:11">
+    <row r="47" spans="1:11" ht="36">
       <c r="A47" s="2"/>
       <c r="B47" s="7">
         <f>ROW(B47)-ROW($B$2)</f>
@@ -5054,7 +4462,7 @@
       </c>
       <c r="K47" s="9"/>
     </row>
-    <row r="48" ht="15.75" spans="1:11">
+    <row r="48" spans="1:11">
       <c r="A48" s="2"/>
       <c r="B48" s="7">
         <f t="shared" si="0"/>
@@ -5086,7 +4494,7 @@
       </c>
       <c r="K48" s="12"/>
     </row>
-    <row r="49" ht="24.75" spans="1:11">
+    <row r="49" spans="1:11" ht="24">
       <c r="A49" s="2"/>
       <c r="B49" s="7">
         <f>ROW(B49)-ROW($B$2)</f>
@@ -5118,7 +4526,7 @@
       </c>
       <c r="K49" s="9"/>
     </row>
-    <row r="50" ht="15.75" spans="1:11">
+    <row r="50" spans="1:11">
       <c r="A50" s="2"/>
       <c r="B50" s="7">
         <f t="shared" si="0"/>
@@ -5150,7 +4558,7 @@
       </c>
       <c r="K50" s="12"/>
     </row>
-    <row r="51" ht="24.75" spans="1:11">
+    <row r="51" spans="1:11" ht="24">
       <c r="A51" s="2"/>
       <c r="B51" s="7">
         <f>ROW(B51)-ROW($B$2)</f>
@@ -5182,7 +4590,7 @@
       </c>
       <c r="K51" s="9"/>
     </row>
-    <row r="52" ht="24.75" spans="1:11">
+    <row r="52" spans="1:11" ht="24">
       <c r="A52" s="2"/>
       <c r="B52" s="7">
         <f t="shared" si="0"/>
@@ -5214,7 +4622,7 @@
       </c>
       <c r="K52" s="12"/>
     </row>
-    <row r="53" ht="24.75" spans="1:11">
+    <row r="53" spans="1:11" ht="24">
       <c r="A53" s="2"/>
       <c r="B53" s="7">
         <f>ROW(B53)-ROW($B$2)</f>
@@ -5246,7 +4654,7 @@
       </c>
       <c r="K53" s="9"/>
     </row>
-    <row r="54" ht="36.75" spans="1:11">
+    <row r="54" spans="1:11" ht="36">
       <c r="A54" s="2"/>
       <c r="B54" s="7">
         <f t="shared" si="0"/>
@@ -5278,7 +4686,7 @@
       </c>
       <c r="K54" s="12"/>
     </row>
-    <row r="55" ht="24.75" spans="1:11">
+    <row r="55" spans="1:11" ht="24">
       <c r="A55" s="2"/>
       <c r="B55" s="7">
         <f>ROW(B55)-ROW($B$2)</f>
@@ -5310,7 +4718,7 @@
       </c>
       <c r="K55" s="9"/>
     </row>
-    <row r="56" ht="24.75" spans="1:11">
+    <row r="56" spans="1:11" ht="24">
       <c r="A56" s="2"/>
       <c r="B56" s="7">
         <f t="shared" si="0"/>
@@ -5342,7 +4750,7 @@
       </c>
       <c r="K56" s="12"/>
     </row>
-    <row r="57" ht="15.75" spans="1:11">
+    <row r="57" spans="1:11" ht="24">
       <c r="A57" s="2"/>
       <c r="B57" s="7">
         <f>ROW(B57)-ROW($B$2)</f>
@@ -5370,7 +4778,7 @@
       </c>
       <c r="K57" s="9"/>
     </row>
-    <row r="58" ht="24.75" spans="1:11">
+    <row r="58" spans="1:11" ht="36">
       <c r="A58" s="2"/>
       <c r="B58" s="7">
         <f t="shared" si="0"/>
@@ -5402,7 +4810,7 @@
       </c>
       <c r="K58" s="12"/>
     </row>
-    <row r="59" ht="24.75" spans="1:11">
+    <row r="59" spans="1:11" ht="24">
       <c r="A59" s="2"/>
       <c r="B59" s="7">
         <f>ROW(B59)-ROW($B$2)</f>
@@ -5434,7 +4842,7 @@
       </c>
       <c r="K59" s="9"/>
     </row>
-    <row r="60" ht="36.75" spans="1:11">
+    <row r="60" spans="1:11" ht="36">
       <c r="A60" s="2"/>
       <c r="B60" s="7">
         <f t="shared" si="0"/>
@@ -5466,7 +4874,7 @@
       </c>
       <c r="K60" s="12"/>
     </row>
-    <row r="61" ht="15.75" spans="1:11">
+    <row r="61" spans="1:11">
       <c r="A61" s="2"/>
       <c r="B61" s="7">
         <f>ROW(B61)-ROW($B$2)</f>
@@ -5498,7 +4906,7 @@
       </c>
       <c r="K61" s="9"/>
     </row>
-    <row r="62" ht="15.75" spans="1:11">
+    <row r="62" spans="1:11">
       <c r="A62" s="2"/>
       <c r="B62" s="7">
         <f t="shared" si="0"/>
@@ -5530,7 +4938,7 @@
       </c>
       <c r="K62" s="12"/>
     </row>
-    <row r="63" ht="48.75" spans="1:11">
+    <row r="63" spans="1:11" ht="48">
       <c r="A63" s="2"/>
       <c r="B63" s="7">
         <f>ROW(B63)-ROW($B$2)</f>
@@ -5562,7 +4970,7 @@
       </c>
       <c r="K63" s="9"/>
     </row>
-    <row r="64" ht="24.75" spans="1:11">
+    <row r="64" spans="1:11" ht="24">
       <c r="A64" s="2"/>
       <c r="B64" s="7">
         <f t="shared" si="0"/>
@@ -5594,37 +5002,39 @@
       </c>
       <c r="K64" s="12"/>
     </row>
-    <row r="65" ht="15.75" spans="1:11">
+    <row r="65" spans="1:11">
       <c r="A65" s="2"/>
       <c r="B65" s="7">
         <f>ROW(B65)-ROW($B$2)</f>
         <v>63</v>
       </c>
-      <c r="C65" s="8" t="s">
+      <c r="C65" s="23" t="s">
         <v>274</v>
       </c>
-      <c r="D65" s="9" t="s">
+      <c r="D65" s="24" t="s">
         <v>275</v>
       </c>
-      <c r="E65" s="10" t="s">
+      <c r="E65" s="25" t="s">
         <v>276</v>
       </c>
-      <c r="F65" s="9" t="s">
+      <c r="F65" s="24" t="s">
         <v>277</v>
       </c>
-      <c r="G65" s="10" t="s">
+      <c r="G65" s="25" t="s">
         <v>278</v>
       </c>
-      <c r="H65" s="9"/>
-      <c r="I65" s="10" t="s">
+      <c r="H65" s="24"/>
+      <c r="I65" s="25" t="s">
         <v>278</v>
       </c>
-      <c r="J65" s="9">
-        <v>1</v>
-      </c>
-      <c r="K65" s="9"/>
-    </row>
-    <row r="66" ht="48.75" spans="1:11">
+      <c r="J65" s="24">
+        <v>1</v>
+      </c>
+      <c r="K65" s="16" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="48">
       <c r="A66" s="2"/>
       <c r="B66" s="7">
         <f t="shared" si="0"/>
@@ -5656,7 +5066,7 @@
       </c>
       <c r="K66" s="12"/>
     </row>
-    <row r="67" ht="26.25" spans="1:11">
+    <row r="67" spans="1:11" ht="25.5">
       <c r="A67" s="2"/>
       <c r="B67" s="7">
         <f>ROW(B67)-ROW($B$2)</f>
@@ -5688,7 +5098,7 @@
       </c>
       <c r="K67" s="9"/>
     </row>
-    <row r="68" ht="15.75" spans="1:11">
+    <row r="68" spans="1:11" ht="24">
       <c r="A68" s="2"/>
       <c r="B68" s="7">
         <f t="shared" si="0"/>
@@ -5720,7 +5130,7 @@
       </c>
       <c r="K68" s="12"/>
     </row>
-    <row r="69" ht="15.75" spans="1:11">
+    <row r="69" spans="1:11">
       <c r="A69" s="2"/>
       <c r="B69" s="7">
         <f>ROW(B69)-ROW($B$2)</f>
@@ -5752,7 +5162,7 @@
       </c>
       <c r="K69" s="9"/>
     </row>
-    <row r="70" ht="36.75" spans="1:11">
+    <row r="70" spans="1:11" ht="36">
       <c r="A70" s="2"/>
       <c r="B70" s="7">
         <f t="shared" si="0"/>
@@ -5784,7 +5194,7 @@
       </c>
       <c r="K70" s="12"/>
     </row>
-    <row r="71" ht="24.75" spans="1:11">
+    <row r="71" spans="1:11" ht="24">
       <c r="A71" s="2"/>
       <c r="B71" s="7">
         <f>ROW(B71)-ROW($B$2)</f>
@@ -5816,7 +5226,7 @@
       </c>
       <c r="K71" s="9"/>
     </row>
-    <row r="72" ht="36.75" spans="1:11">
+    <row r="72" spans="1:11" ht="36">
       <c r="A72" s="2"/>
       <c r="B72" s="7">
         <f t="shared" si="0"/>
@@ -5848,7 +5258,7 @@
       </c>
       <c r="K72" s="12"/>
     </row>
-    <row r="73" ht="24.75" spans="1:11">
+    <row r="73" spans="1:11" ht="24">
       <c r="A73" s="2"/>
       <c r="B73" s="7">
         <f>ROW(B73)-ROW($B$2)</f>
@@ -5880,7 +5290,7 @@
       </c>
       <c r="K73" s="9"/>
     </row>
-    <row r="74" ht="24.75" spans="1:11">
+    <row r="74" spans="1:11" ht="24">
       <c r="A74" s="2"/>
       <c r="B74" s="7">
         <f t="shared" si="0"/>
@@ -5912,7 +5322,7 @@
       </c>
       <c r="K74" s="12"/>
     </row>
-    <row r="75" ht="24.75" spans="1:11">
+    <row r="75" spans="1:11" ht="24">
       <c r="A75" s="2"/>
       <c r="B75" s="7">
         <f>ROW(B75)-ROW($B$2)</f>
@@ -5944,7 +5354,7 @@
       </c>
       <c r="K75" s="9"/>
     </row>
-    <row r="76" ht="24.75" spans="1:11">
+    <row r="76" spans="1:11" ht="24">
       <c r="A76" s="2"/>
       <c r="B76" s="7">
         <f t="shared" si="0"/>
@@ -5976,7 +5386,7 @@
       </c>
       <c r="K76" s="12"/>
     </row>
-    <row r="77" ht="15.75" spans="1:11">
+    <row r="77" spans="1:11">
       <c r="A77" s="2"/>
       <c r="B77" s="7">
         <f>ROW(B77)-ROW($B$2)</f>
@@ -6008,7 +5418,7 @@
       </c>
       <c r="K77" s="9"/>
     </row>
-    <row r="78" ht="24.75" spans="1:11">
+    <row r="78" spans="1:11" ht="24">
       <c r="A78" s="2"/>
       <c r="B78" s="7">
         <f t="shared" si="0"/>
@@ -6040,7 +5450,7 @@
       </c>
       <c r="K78" s="12"/>
     </row>
-    <row r="79" ht="15.75" spans="1:11">
+    <row r="79" spans="1:11">
       <c r="A79" s="2"/>
       <c r="B79" s="7">
         <f>ROW(B79)-ROW($B$2)</f>
@@ -6070,7 +5480,7 @@
       </c>
       <c r="K79" s="9"/>
     </row>
-    <row r="80" ht="24.75" spans="1:11">
+    <row r="80" spans="1:11" ht="24">
       <c r="A80" s="2"/>
       <c r="B80" s="7">
         <f t="shared" si="0"/>
@@ -6102,7 +5512,7 @@
       </c>
       <c r="K80" s="12"/>
     </row>
-    <row r="81" ht="24.75" spans="1:11">
+    <row r="81" spans="1:11" ht="24">
       <c r="A81" s="2"/>
       <c r="B81" s="7">
         <f>ROW(B81)-ROW($B$2)</f>
@@ -6134,7 +5544,7 @@
       </c>
       <c r="K81" s="9"/>
     </row>
-    <row r="82" ht="24.75" spans="1:11">
+    <row r="82" spans="1:11" ht="24">
       <c r="A82" s="2"/>
       <c r="B82" s="7">
         <f t="shared" si="0"/>
@@ -6166,7 +5576,7 @@
       </c>
       <c r="K82" s="12"/>
     </row>
-    <row r="83" ht="24.75" spans="1:11">
+    <row r="83" spans="1:11" ht="24">
       <c r="A83" s="2"/>
       <c r="B83" s="7">
         <f>ROW(B83)-ROW($B$2)</f>
@@ -6198,7 +5608,7 @@
       </c>
       <c r="K83" s="9"/>
     </row>
-    <row r="84" ht="24.75" spans="1:11">
+    <row r="84" spans="1:11" ht="24">
       <c r="A84" s="2"/>
       <c r="B84" s="7">
         <f t="shared" si="0"/>
@@ -6230,7 +5640,7 @@
       </c>
       <c r="K84" s="12"/>
     </row>
-    <row r="85" ht="48.75" spans="1:11">
+    <row r="85" spans="1:11" ht="48">
       <c r="A85" s="2"/>
       <c r="B85" s="7">
         <f>ROW(B85)-ROW($B$2)</f>
@@ -6262,7 +5672,7 @@
       </c>
       <c r="K85" s="9"/>
     </row>
-    <row r="86" ht="24.75" spans="1:11">
+    <row r="86" spans="1:11" ht="24">
       <c r="A86" s="2"/>
       <c r="B86" s="7">
         <f t="shared" si="0"/>
@@ -6294,7 +5704,7 @@
       </c>
       <c r="K86" s="12"/>
     </row>
-    <row r="87" ht="24.75" spans="1:11">
+    <row r="87" spans="1:11" ht="24">
       <c r="A87" s="2"/>
       <c r="B87" s="7">
         <f>ROW(B87)-ROW($B$2)</f>
@@ -6326,7 +5736,7 @@
       </c>
       <c r="K87" s="9"/>
     </row>
-    <row r="88" ht="24.75" spans="1:11">
+    <row r="88" spans="1:11" ht="24">
       <c r="A88" s="2"/>
       <c r="B88" s="7">
         <f t="shared" si="0"/>
@@ -6358,7 +5768,7 @@
       </c>
       <c r="K88" s="12"/>
     </row>
-    <row r="89" ht="24.75" spans="1:11">
+    <row r="89" spans="1:11" ht="24">
       <c r="A89" s="2"/>
       <c r="B89" s="7">
         <f>ROW(B89)-ROW($B$2)</f>
@@ -6388,7 +5798,7 @@
       </c>
       <c r="K89" s="9"/>
     </row>
-    <row r="90" ht="15.75" spans="1:11">
+    <row r="90" spans="1:11">
       <c r="A90" s="2"/>
       <c r="B90" s="7">
         <f t="shared" si="0"/>
@@ -6397,30 +5807,30 @@
       <c r="C90" s="11" t="s">
         <v>394</v>
       </c>
-      <c r="D90" s="18" t="s">
+      <c r="D90" s="17" t="s">
         <v>395</v>
       </c>
-      <c r="E90" s="19" t="s">
+      <c r="E90" s="18" t="s">
         <v>396</v>
       </c>
-      <c r="F90" s="18" t="s">
+      <c r="F90" s="17" t="s">
         <v>391</v>
       </c>
-      <c r="G90" s="19" t="s">
+      <c r="G90" s="18" t="s">
         <v>397</v>
       </c>
-      <c r="H90" s="18" t="s">
+      <c r="H90" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="I90" s="19" t="s">
+      <c r="I90" s="18" t="s">
         <v>398</v>
       </c>
-      <c r="J90" s="18">
-        <v>1</v>
-      </c>
-      <c r="K90" s="17"/>
-    </row>
-    <row r="91" ht="15.75" spans="1:11">
+      <c r="J90" s="17">
+        <v>1</v>
+      </c>
+      <c r="K90" s="16"/>
+    </row>
+    <row r="91" spans="1:11">
       <c r="A91" s="2"/>
       <c r="B91" s="7">
         <f>ROW(B91)-ROW($B$2)</f>
@@ -6450,7 +5860,7 @@
       </c>
       <c r="K91" s="9"/>
     </row>
-    <row r="92" ht="84.75" spans="1:11">
+    <row r="92" spans="1:11" ht="96">
       <c r="A92" s="2"/>
       <c r="B92" s="7">
         <f t="shared" si="0"/>
@@ -6482,7 +5892,7 @@
       </c>
       <c r="K92" s="12"/>
     </row>
-    <row r="93" ht="15.75" spans="1:11">
+    <row r="93" spans="1:11">
       <c r="A93" s="2"/>
       <c r="B93" s="7">
         <f>ROW(B93)-ROW($B$2)</f>
@@ -6514,7 +5924,7 @@
       </c>
       <c r="K93" s="9"/>
     </row>
-    <row r="94" ht="15.75" spans="1:11">
+    <row r="94" spans="1:11">
       <c r="A94" s="2"/>
       <c r="B94" s="7">
         <f t="shared" si="0"/>
@@ -6546,7 +5956,7 @@
       </c>
       <c r="K94" s="12"/>
     </row>
-    <row r="95" ht="15.75" spans="1:11">
+    <row r="95" spans="1:11">
       <c r="A95" s="2"/>
       <c r="B95" s="7">
         <f>ROW(B95)-ROW($B$2)</f>
@@ -6578,7 +5988,7 @@
       </c>
       <c r="K95" s="9"/>
     </row>
-    <row r="96" ht="15.75" spans="1:11">
+    <row r="96" spans="1:11">
       <c r="A96" s="2"/>
       <c r="B96" s="7">
         <f t="shared" si="0"/>
@@ -6610,7 +6020,7 @@
       </c>
       <c r="K96" s="12"/>
     </row>
-    <row r="97" ht="15.75" spans="1:11">
+    <row r="97" spans="1:11">
       <c r="A97" s="2"/>
       <c r="B97" s="7">
         <f>ROW(B97)-ROW($B$2)</f>
@@ -6642,7 +6052,7 @@
       </c>
       <c r="K97" s="9"/>
     </row>
-    <row r="98" ht="15.75" spans="1:11">
+    <row r="98" spans="1:11">
       <c r="A98" s="2"/>
       <c r="B98" s="7">
         <f t="shared" si="0"/>
@@ -6674,7 +6084,7 @@
       </c>
       <c r="K98" s="12"/>
     </row>
-    <row r="99" ht="15.75" spans="1:11">
+    <row r="99" spans="1:11">
       <c r="A99" s="2"/>
       <c r="B99" s="7">
         <f>ROW(B99)-ROW($B$2)</f>
@@ -6706,7 +6116,7 @@
       </c>
       <c r="K99" s="9"/>
     </row>
-    <row r="100" ht="24.75" spans="1:11">
+    <row r="100" spans="1:11" ht="24">
       <c r="A100" s="2"/>
       <c r="B100" s="7">
         <f t="shared" si="0"/>
@@ -6738,7 +6148,7 @@
       </c>
       <c r="K100" s="12"/>
     </row>
-    <row r="101" ht="15.75" spans="1:11">
+    <row r="101" spans="1:11">
       <c r="A101" s="2"/>
       <c r="B101" s="7">
         <f>ROW(B101)-ROW($B$2)</f>
@@ -6770,7 +6180,7 @@
       </c>
       <c r="K101" s="9"/>
     </row>
-    <row r="102" ht="15.75" spans="1:11">
+    <row r="102" spans="1:11">
       <c r="A102" s="2"/>
       <c r="B102" s="7">
         <f t="shared" si="0"/>
@@ -6802,7 +6212,7 @@
       </c>
       <c r="K102" s="12"/>
     </row>
-    <row r="103" ht="36.75" spans="1:11">
+    <row r="103" spans="1:11" ht="36">
       <c r="A103" s="2"/>
       <c r="B103" s="7">
         <f>ROW(B103)-ROW($B$2)</f>
@@ -6834,7 +6244,7 @@
       </c>
       <c r="K103" s="9"/>
     </row>
-    <row r="104" ht="15.75" spans="1:11">
+    <row r="104" spans="1:11">
       <c r="A104" s="2"/>
       <c r="B104" s="7">
         <f t="shared" si="0"/>
@@ -6866,7 +6276,7 @@
       </c>
       <c r="K104" s="12"/>
     </row>
-    <row r="105" ht="15.75" spans="1:11">
+    <row r="105" spans="1:11">
       <c r="A105" s="2"/>
       <c r="B105" s="7">
         <f>ROW(B105)-ROW($B$2)</f>
@@ -6898,7 +6308,7 @@
       </c>
       <c r="K105" s="9"/>
     </row>
-    <row r="106" ht="15.75" spans="1:11">
+    <row r="106" spans="1:11">
       <c r="A106" s="2"/>
       <c r="B106" s="7">
         <f t="shared" si="0"/>
@@ -6930,7 +6340,7 @@
       </c>
       <c r="K106" s="12"/>
     </row>
-    <row r="107" ht="15.75" spans="1:11">
+    <row r="107" spans="1:11">
       <c r="A107" s="2"/>
       <c r="B107" s="7">
         <f>ROW(B107)-ROW($B$2)</f>
@@ -6962,7 +6372,7 @@
       </c>
       <c r="K107" s="9"/>
     </row>
-    <row r="108" ht="15.75" spans="1:11">
+    <row r="108" spans="1:11">
       <c r="A108" s="2"/>
       <c r="B108" s="7">
         <f t="shared" si="0"/>
@@ -6994,7 +6404,7 @@
       </c>
       <c r="K108" s="12"/>
     </row>
-    <row r="109" ht="15.75" spans="1:11">
+    <row r="109" spans="1:11">
       <c r="A109" s="2"/>
       <c r="B109" s="7">
         <f>ROW(B109)-ROW($B$2)</f>
@@ -7026,7 +6436,7 @@
       </c>
       <c r="K109" s="9"/>
     </row>
-    <row r="110" ht="15.75" spans="1:11">
+    <row r="110" spans="1:11" ht="24">
       <c r="A110" s="2"/>
       <c r="B110" s="7">
         <f t="shared" si="0"/>
@@ -7056,7 +6466,7 @@
       </c>
       <c r="K110" s="12"/>
     </row>
-    <row r="111" ht="15.75" spans="1:11">
+    <row r="111" spans="1:11">
       <c r="A111" s="2"/>
       <c r="B111" s="7">
         <f>ROW(B111)-ROW($B$2)</f>
@@ -7088,7 +6498,7 @@
       </c>
       <c r="K111" s="9"/>
     </row>
-    <row r="112" ht="15.75" spans="1:11">
+    <row r="112" spans="1:11">
       <c r="A112" s="2"/>
       <c r="B112" s="7">
         <f t="shared" si="0"/>
@@ -7120,7 +6530,7 @@
       </c>
       <c r="K112" s="12"/>
     </row>
-    <row r="113" ht="15.75" spans="1:11">
+    <row r="113" spans="1:11">
       <c r="A113" s="2"/>
       <c r="B113" s="7">
         <f>ROW(B113)-ROW($B$2)</f>
@@ -7152,7 +6562,7 @@
       </c>
       <c r="K113" s="9"/>
     </row>
-    <row r="114" ht="15.75" spans="1:11">
+    <row r="114" spans="1:11">
       <c r="A114" s="2"/>
       <c r="B114" s="7">
         <f t="shared" si="0"/>
@@ -7182,11 +6592,11 @@
       <c r="J114" s="14">
         <v>1</v>
       </c>
-      <c r="K114" s="17" t="s">
+      <c r="K114" s="16" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="115" ht="15.75" spans="1:11">
+    <row r="115" spans="1:11" ht="24">
       <c r="A115" s="2"/>
       <c r="B115" s="7">
         <f>ROW(B115)-ROW($B$2)</f>
@@ -7216,7 +6626,7 @@
       </c>
       <c r="K115" s="9"/>
     </row>
-    <row r="116" ht="15.75" spans="1:11">
+    <row r="116" spans="1:11">
       <c r="A116" s="2"/>
       <c r="B116" s="7">
         <f t="shared" si="0"/>
@@ -7248,7 +6658,7 @@
       </c>
       <c r="K116" s="12"/>
     </row>
-    <row r="117" ht="15.75" spans="1:11">
+    <row r="117" spans="1:11">
       <c r="A117" s="2"/>
       <c r="B117" s="7">
         <f>ROW(B117)-ROW($B$2)</f>
@@ -7280,7 +6690,7 @@
       </c>
       <c r="K117" s="9"/>
     </row>
-    <row r="118" ht="15.75" spans="1:11">
+    <row r="118" spans="1:11">
       <c r="A118" s="2"/>
       <c r="B118" s="7">
         <f t="shared" si="0"/>
@@ -7312,7 +6722,7 @@
       </c>
       <c r="K118" s="12"/>
     </row>
-    <row r="119" ht="15.75" spans="1:11">
+    <row r="119" spans="1:11">
       <c r="A119" s="2"/>
       <c r="B119" s="7">
         <f>ROW(B119)-ROW($B$2)</f>
@@ -7344,7 +6754,7 @@
       </c>
       <c r="K119" s="9"/>
     </row>
-    <row r="120" ht="15.75" spans="1:11">
+    <row r="120" spans="1:11">
       <c r="A120" s="2"/>
       <c r="B120" s="7">
         <f t="shared" si="0"/>
@@ -7374,7 +6784,7 @@
       </c>
       <c r="K120" s="12"/>
     </row>
-    <row r="121" ht="36.75" spans="1:11">
+    <row r="121" spans="1:11" ht="36">
       <c r="A121" s="2"/>
       <c r="B121" s="7">
         <f>ROW(B121)-ROW($B$2)</f>
@@ -7402,7 +6812,7 @@
       </c>
       <c r="K121" s="9"/>
     </row>
-    <row r="122" ht="15.75" spans="1:11">
+    <row r="122" spans="1:11">
       <c r="A122" s="2"/>
       <c r="B122" s="7">
         <f t="shared" si="0"/>
@@ -7432,7 +6842,7 @@
       </c>
       <c r="K122" s="12"/>
     </row>
-    <row r="123" ht="24.75" spans="1:11">
+    <row r="123" spans="1:11" ht="24">
       <c r="A123" s="2"/>
       <c r="B123" s="7">
         <f>ROW(B123)-ROW($B$2)</f>
@@ -7464,7 +6874,7 @@
       </c>
       <c r="K123" s="9"/>
     </row>
-    <row r="124" ht="15.75" spans="1:11">
+    <row r="124" spans="1:11">
       <c r="A124" s="2"/>
       <c r="B124" s="7">
         <f t="shared" si="0"/>
@@ -7496,7 +6906,7 @@
       </c>
       <c r="K124" s="12"/>
     </row>
-    <row r="125" ht="15.75" spans="1:11">
+    <row r="125" spans="1:11">
       <c r="A125" s="2"/>
       <c r="B125" s="7">
         <f>ROW(B125)-ROW($B$2)</f>
@@ -7528,7 +6938,7 @@
       </c>
       <c r="K125" s="9"/>
     </row>
-    <row r="126" ht="15.75" spans="1:11">
+    <row r="126" spans="1:11">
       <c r="A126" s="2"/>
       <c r="B126" s="7">
         <f t="shared" si="0"/>
@@ -7556,11 +6966,11 @@
       <c r="J126" s="14">
         <v>1</v>
       </c>
-      <c r="K126" s="17" t="s">
+      <c r="K126" s="16" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="127" ht="15.75" spans="1:11">
+    <row r="127" spans="1:11">
       <c r="A127" s="2"/>
       <c r="B127" s="7">
         <f>ROW(B127)-ROW($B$2)</f>
@@ -7592,7 +7002,7 @@
       </c>
       <c r="K127" s="9"/>
     </row>
-    <row r="128" ht="15.75" spans="1:11">
+    <row r="128" spans="1:11">
       <c r="A128" s="2"/>
       <c r="B128" s="7">
         <f t="shared" si="0"/>
@@ -7624,7 +7034,7 @@
       </c>
       <c r="K128" s="12"/>
     </row>
-    <row r="129" ht="15.75" spans="1:11">
+    <row r="129" spans="1:11">
       <c r="A129" s="2"/>
       <c r="B129" s="7">
         <f>ROW(B129)-ROW($B$2)</f>
@@ -7656,7 +7066,7 @@
       </c>
       <c r="K129" s="9"/>
     </row>
-    <row r="130" ht="15.75" spans="1:11">
+    <row r="130" spans="1:11">
       <c r="A130" s="2"/>
       <c r="B130" s="7">
         <f t="shared" si="0"/>
@@ -7686,7 +7096,7 @@
       </c>
       <c r="K130" s="12"/>
     </row>
-    <row r="131" ht="15.75" spans="1:11">
+    <row r="131" spans="1:11">
       <c r="A131" s="2"/>
       <c r="B131" s="7">
         <f>ROW(B131)-ROW($B$2)</f>
@@ -7718,7 +7128,7 @@
       </c>
       <c r="K131" s="9"/>
     </row>
-    <row r="132" ht="15.75" spans="1:11">
+    <row r="132" spans="1:11">
       <c r="A132" s="2"/>
       <c r="B132" s="7">
         <f t="shared" si="0"/>
@@ -7750,7 +7160,7 @@
       </c>
       <c r="K132" s="12"/>
     </row>
-    <row r="133" ht="15.75" spans="1:11">
+    <row r="133" spans="1:11">
       <c r="A133" s="2"/>
       <c r="B133" s="7">
         <f>ROW(B133)-ROW($B$2)</f>
@@ -7780,7 +7190,7 @@
       </c>
       <c r="K133" s="9"/>
     </row>
-    <row r="134" ht="15.75" spans="1:11">
+    <row r="134" spans="1:11">
       <c r="A134" s="2"/>
       <c r="B134" s="7">
         <f t="shared" si="0"/>
@@ -7812,7 +7222,7 @@
       </c>
       <c r="K134" s="12"/>
     </row>
-    <row r="135" ht="15.75" spans="1:11">
+    <row r="135" spans="1:11" ht="24">
       <c r="A135" s="2"/>
       <c r="B135" s="7">
         <f>ROW(B135)-ROW($B$2)</f>
@@ -7842,7 +7252,7 @@
       </c>
       <c r="K135" s="9"/>
     </row>
-    <row r="136" ht="15.75" spans="1:11">
+    <row r="136" spans="1:11">
       <c r="A136" s="2"/>
       <c r="B136" s="7">
         <f t="shared" si="0"/>
@@ -7874,7 +7284,7 @@
       </c>
       <c r="K136" s="12"/>
     </row>
-    <row r="137" ht="15.75" spans="1:11">
+    <row r="137" spans="1:11">
       <c r="A137" s="2"/>
       <c r="B137" s="7">
         <f>ROW(B137)-ROW($B$2)</f>
@@ -7906,7 +7316,7 @@
       </c>
       <c r="K137" s="9"/>
     </row>
-    <row r="138" ht="15.75" spans="1:11">
+    <row r="138" spans="1:11">
       <c r="A138" s="2"/>
       <c r="B138" s="7">
         <f t="shared" si="0"/>
@@ -7938,7 +7348,7 @@
       </c>
       <c r="K138" s="12"/>
     </row>
-    <row r="139" ht="15.75" spans="1:11">
+    <row r="139" spans="1:11">
       <c r="A139" s="2"/>
       <c r="B139" s="7">
         <f>ROW(B139)-ROW($B$2)</f>
@@ -7970,7 +7380,7 @@
       </c>
       <c r="K139" s="9"/>
     </row>
-    <row r="140" ht="15.75" spans="1:11">
+    <row r="140" spans="1:11">
       <c r="A140" s="2"/>
       <c r="B140" s="7">
         <f t="shared" si="0"/>
@@ -8000,7 +7410,7 @@
       </c>
       <c r="K140" s="12"/>
     </row>
-    <row r="141" ht="15.75" spans="1:11">
+    <row r="141" spans="1:11">
       <c r="A141" s="2"/>
       <c r="B141" s="7">
         <f>ROW(B141)-ROW($B$2)</f>
@@ -8032,7 +7442,7 @@
       </c>
       <c r="K141" s="9"/>
     </row>
-    <row r="142" ht="15.75" spans="1:11">
+    <row r="142" spans="1:11">
       <c r="A142" s="2"/>
       <c r="B142" s="7">
         <f t="shared" si="0"/>
@@ -8062,7 +7472,7 @@
       </c>
       <c r="K142" s="12"/>
     </row>
-    <row r="143" ht="15.75" spans="1:11">
+    <row r="143" spans="1:11">
       <c r="A143" s="2"/>
       <c r="B143" s="7">
         <f>ROW(B143)-ROW($B$2)</f>
@@ -8094,7 +7504,7 @@
       </c>
       <c r="K143" s="9"/>
     </row>
-    <row r="144" ht="15.75" spans="1:11">
+    <row r="144" spans="1:11">
       <c r="A144" s="2"/>
       <c r="B144" s="7">
         <f t="shared" si="0"/>
@@ -8124,7 +7534,7 @@
       </c>
       <c r="K144" s="12"/>
     </row>
-    <row r="145" ht="15.75" spans="1:11">
+    <row r="145" spans="1:11">
       <c r="A145" s="2"/>
       <c r="B145" s="7">
         <f>ROW(B145)-ROW($B$2)</f>
@@ -8156,7 +7566,7 @@
       </c>
       <c r="K145" s="9"/>
     </row>
-    <row r="146" ht="15.75" spans="1:11">
+    <row r="146" spans="1:11">
       <c r="A146" s="2"/>
       <c r="B146" s="7">
         <f t="shared" si="0"/>
@@ -8188,7 +7598,7 @@
       </c>
       <c r="K146" s="12"/>
     </row>
-    <row r="147" ht="15.75" spans="1:11">
+    <row r="147" spans="1:11">
       <c r="A147" s="2"/>
       <c r="B147" s="7">
         <f>ROW(B147)-ROW($B$2)</f>
@@ -8220,7 +7630,7 @@
       </c>
       <c r="K147" s="9"/>
     </row>
-    <row r="148" ht="15.75" spans="1:11">
+    <row r="148" spans="1:11">
       <c r="A148" s="2"/>
       <c r="B148" s="7">
         <f t="shared" si="0"/>
@@ -8252,7 +7662,7 @@
       </c>
       <c r="K148" s="12"/>
     </row>
-    <row r="149" ht="15.75" spans="1:11">
+    <row r="149" spans="1:11">
       <c r="A149" s="2"/>
       <c r="B149" s="7">
         <f>ROW(B149)-ROW($B$2)</f>
@@ -8284,7 +7694,7 @@
       </c>
       <c r="K149" s="9"/>
     </row>
-    <row r="150" ht="15.75" spans="1:11">
+    <row r="150" spans="1:11">
       <c r="A150" s="2"/>
       <c r="B150" s="7">
         <f t="shared" si="0"/>
@@ -8316,7 +7726,7 @@
       </c>
       <c r="K150" s="12"/>
     </row>
-    <row r="151" ht="15.75" spans="1:11">
+    <row r="151" spans="1:11">
       <c r="A151" s="2"/>
       <c r="B151" s="7">
         <f>ROW(B151)-ROW($B$2)</f>
@@ -8348,7 +7758,7 @@
       </c>
       <c r="K151" s="9"/>
     </row>
-    <row r="152" ht="15.75" spans="1:11">
+    <row r="152" spans="1:11">
       <c r="A152" s="2"/>
       <c r="B152" s="7">
         <f t="shared" si="0"/>
@@ -8380,7 +7790,7 @@
       </c>
       <c r="K152" s="12"/>
     </row>
-    <row r="153" ht="15.75" spans="1:11">
+    <row r="153" spans="1:11">
       <c r="A153" s="2"/>
       <c r="B153" s="7">
         <f>ROW(B153)-ROW($B$2)</f>
@@ -8412,7 +7822,7 @@
       </c>
       <c r="K153" s="9"/>
     </row>
-    <row r="154" ht="15.75" spans="1:11">
+    <row r="154" spans="1:11">
       <c r="A154" s="2"/>
       <c r="B154" s="7">
         <f t="shared" si="0"/>
@@ -8444,7 +7854,7 @@
       </c>
       <c r="K154" s="12"/>
     </row>
-    <row r="155" ht="15.75" spans="1:11">
+    <row r="155" spans="1:11">
       <c r="A155" s="2"/>
       <c r="B155" s="7">
         <f>ROW(B155)-ROW($B$2)</f>
@@ -8476,7 +7886,7 @@
       </c>
       <c r="K155" s="9"/>
     </row>
-    <row r="156" ht="15.75" spans="1:11">
+    <row r="156" spans="1:11">
       <c r="A156" s="2"/>
       <c r="B156" s="7">
         <f t="shared" si="0"/>
@@ -8508,7 +7918,7 @@
       </c>
       <c r="K156" s="12"/>
     </row>
-    <row r="157" ht="15.75" spans="1:11">
+    <row r="157" spans="1:11">
       <c r="A157" s="2"/>
       <c r="B157" s="7">
         <f>ROW(B157)-ROW($B$2)</f>
@@ -8540,7 +7950,7 @@
       </c>
       <c r="K157" s="9"/>
     </row>
-    <row r="158" ht="24.75" spans="1:11">
+    <row r="158" spans="1:11" ht="24">
       <c r="A158" s="2"/>
       <c r="B158" s="7">
         <f t="shared" si="0"/>
@@ -8572,7 +7982,7 @@
       </c>
       <c r="K158" s="12"/>
     </row>
-    <row r="159" ht="24.75" spans="1:11">
+    <row r="159" spans="1:11" ht="24">
       <c r="A159" s="2"/>
       <c r="B159" s="7">
         <f>ROW(B159)-ROW($B$2)</f>
@@ -8602,7 +8012,7 @@
       </c>
       <c r="K159" s="9"/>
     </row>
-    <row r="160" ht="24.75" spans="1:11">
+    <row r="160" spans="1:11" ht="24">
       <c r="A160" s="2"/>
       <c r="B160" s="7">
         <f t="shared" si="0"/>
@@ -8634,7 +8044,7 @@
       </c>
       <c r="K160" s="12"/>
     </row>
-    <row r="161" ht="15.75" spans="1:11">
+    <row r="161" spans="1:11">
       <c r="A161" s="2"/>
       <c r="B161" s="7">
         <f>ROW(B161)-ROW($B$2)</f>
@@ -8666,7 +8076,7 @@
       </c>
       <c r="K161" s="9"/>
     </row>
-    <row r="162" ht="24.75" spans="1:11">
+    <row r="162" spans="1:11" ht="24">
       <c r="A162" s="2"/>
       <c r="B162" s="7">
         <f t="shared" si="0"/>
@@ -8698,7 +8108,7 @@
       </c>
       <c r="K162" s="12"/>
     </row>
-    <row r="163" ht="24.75" spans="1:11">
+    <row r="163" spans="1:11" ht="24">
       <c r="A163" s="2"/>
       <c r="B163" s="7">
         <f>ROW(B163)-ROW($B$2)</f>
@@ -8730,7 +8140,7 @@
       </c>
       <c r="K163" s="9"/>
     </row>
-    <row r="164" ht="15.75" spans="1:11">
+    <row r="164" spans="1:11">
       <c r="A164" s="2"/>
       <c r="B164" s="7">
         <f t="shared" si="0"/>
@@ -8762,7 +8172,7 @@
       </c>
       <c r="K164" s="12"/>
     </row>
-    <row r="165" ht="15.75" spans="1:11">
+    <row r="165" spans="1:11">
       <c r="A165" s="2"/>
       <c r="B165" s="7">
         <f>ROW(B165)-ROW($B$2)</f>
@@ -8794,7 +8204,7 @@
       </c>
       <c r="K165" s="9"/>
     </row>
-    <row r="166" ht="15.75" spans="1:11">
+    <row r="166" spans="1:11">
       <c r="A166" s="2"/>
       <c r="B166" s="7">
         <f t="shared" si="0"/>
@@ -8826,7 +8236,7 @@
       </c>
       <c r="K166" s="12"/>
     </row>
-    <row r="167" ht="15.75" spans="1:11">
+    <row r="167" spans="1:11">
       <c r="A167" s="2"/>
       <c r="B167" s="7">
         <f>ROW(B167)-ROW($B$2)</f>
@@ -8858,7 +8268,7 @@
       </c>
       <c r="K167" s="9"/>
     </row>
-    <row r="168" ht="15.75" spans="1:11">
+    <row r="168" spans="1:11">
       <c r="A168" s="2"/>
       <c r="B168" s="7">
         <f t="shared" si="0"/>
@@ -8890,7 +8300,7 @@
       </c>
       <c r="K168" s="12"/>
     </row>
-    <row r="169" ht="24.75" spans="1:11">
+    <row r="169" spans="1:11" ht="24">
       <c r="A169" s="2"/>
       <c r="B169" s="7">
         <f>ROW(B169)-ROW($B$2)</f>
@@ -8922,7 +8332,7 @@
       </c>
       <c r="K169" s="9"/>
     </row>
-    <row r="170" ht="24.75" spans="1:11">
+    <row r="170" spans="1:11" ht="24">
       <c r="A170" s="2"/>
       <c r="B170" s="7">
         <f t="shared" si="0"/>
@@ -8954,7 +8364,7 @@
       </c>
       <c r="K170" s="12"/>
     </row>
-    <row r="171" ht="24.75" spans="1:11">
+    <row r="171" spans="1:11" ht="24">
       <c r="A171" s="2"/>
       <c r="B171" s="7">
         <f>ROW(B171)-ROW($B$2)</f>
@@ -8986,7 +8396,7 @@
       </c>
       <c r="K171" s="9"/>
     </row>
-    <row r="172" ht="15.75" spans="1:11">
+    <row r="172" spans="1:11">
       <c r="A172" s="2"/>
       <c r="B172" s="7">
         <f t="shared" si="0"/>
@@ -9018,7 +8428,7 @@
       </c>
       <c r="K172" s="12"/>
     </row>
-    <row r="173" ht="15.75" spans="1:11">
+    <row r="173" spans="1:11" ht="24">
       <c r="A173" s="2"/>
       <c r="B173" s="7">
         <f>ROW(B173)-ROW($B$2)</f>
@@ -9050,7 +8460,7 @@
       </c>
       <c r="K173" s="9"/>
     </row>
-    <row r="174" ht="24.75" spans="1:11">
+    <row r="174" spans="1:11" ht="24">
       <c r="A174" s="2"/>
       <c r="B174" s="7">
         <f t="shared" si="0"/>
@@ -9080,7 +8490,7 @@
       </c>
       <c r="K174" s="12"/>
     </row>
-    <row r="175" ht="15.75" spans="1:11">
+    <row r="175" spans="1:11">
       <c r="A175" s="2"/>
       <c r="B175" s="7">
         <f>ROW(B175)-ROW($B$2)</f>
@@ -9112,7 +8522,7 @@
       </c>
       <c r="K175" s="9"/>
     </row>
-    <row r="176" ht="15.75" spans="1:11">
+    <row r="176" spans="1:11">
       <c r="A176" s="2"/>
       <c r="B176" s="7">
         <f t="shared" si="0"/>
@@ -9144,7 +8554,7 @@
       </c>
       <c r="K176" s="12"/>
     </row>
-    <row r="177" ht="36.75" spans="1:11">
+    <row r="177" spans="1:11" ht="36">
       <c r="A177" s="2"/>
       <c r="B177" s="7">
         <f>ROW(B177)-ROW($B$2)</f>
@@ -9176,7 +8586,7 @@
       </c>
       <c r="K177" s="9"/>
     </row>
-    <row r="178" ht="15.75" spans="1:11">
+    <row r="178" spans="1:11">
       <c r="A178" s="2"/>
       <c r="B178" s="7">
         <f t="shared" si="0"/>
@@ -9208,7 +8618,7 @@
       </c>
       <c r="K178" s="12"/>
     </row>
-    <row r="179" ht="15.75" spans="1:11">
+    <row r="179" spans="1:11">
       <c r="A179" s="2"/>
       <c r="B179" s="7">
         <f>ROW(B179)-ROW($B$2)</f>
@@ -9240,7 +8650,7 @@
       </c>
       <c r="K179" s="9"/>
     </row>
-    <row r="180" ht="15.75" spans="1:11">
+    <row r="180" spans="1:11">
       <c r="A180" s="2"/>
       <c r="B180" s="7">
         <f t="shared" si="0"/>
@@ -9272,7 +8682,7 @@
       </c>
       <c r="K180" s="12"/>
     </row>
-    <row r="181" ht="24.75" spans="1:11">
+    <row r="181" spans="1:11" ht="24">
       <c r="A181" s="2"/>
       <c r="B181" s="7">
         <f>ROW(B181)-ROW($B$2)</f>
@@ -9304,7 +8714,7 @@
       </c>
       <c r="K181" s="9"/>
     </row>
-    <row r="182" ht="24.75" spans="1:11">
+    <row r="182" spans="1:11" ht="24">
       <c r="A182" s="2"/>
       <c r="B182" s="7">
         <f t="shared" si="0"/>
@@ -9336,7 +8746,7 @@
       </c>
       <c r="K182" s="12"/>
     </row>
-    <row r="183" ht="24.75" spans="1:11">
+    <row r="183" spans="1:11" ht="24">
       <c r="A183" s="2"/>
       <c r="B183" s="7">
         <f>ROW(B183)-ROW($B$2)</f>
@@ -9368,7 +8778,7 @@
       </c>
       <c r="K183" s="9"/>
     </row>
-    <row r="184" ht="36.75" spans="1:11">
+    <row r="184" spans="1:11" ht="36">
       <c r="A184" s="2"/>
       <c r="B184" s="7">
         <f t="shared" si="0"/>
@@ -9398,105 +8808,104 @@
       </c>
       <c r="K184" s="12"/>
     </row>
-    <row r="185" ht="36.75" spans="2:11">
-      <c r="B185" s="20">
+    <row r="185" spans="1:11" ht="36">
+      <c r="B185" s="19">
         <f>ROW(B185)-ROW($B$2)</f>
         <v>183</v>
       </c>
-      <c r="C185" s="21" t="s">
+      <c r="C185" s="20" t="s">
         <v>776</v>
       </c>
-      <c r="D185" s="22" t="s">
+      <c r="D185" s="21" t="s">
         <v>777</v>
       </c>
-      <c r="E185" s="22" t="s">
+      <c r="E185" s="21" t="s">
         <v>778</v>
       </c>
-      <c r="F185" s="22" t="s">
+      <c r="F185" s="21" t="s">
         <v>779</v>
       </c>
-      <c r="G185" s="22" t="s">
+      <c r="G185" s="21" t="s">
         <v>780</v>
       </c>
-      <c r="H185" s="22" t="s">
+      <c r="H185" s="21" t="s">
         <v>781</v>
       </c>
-      <c r="I185" s="22" t="s">
+      <c r="I185" s="21" t="s">
         <v>782</v>
       </c>
-      <c r="J185" s="22">
-        <v>1</v>
-      </c>
-      <c r="K185" s="22"/>
-    </row>
-    <row r="186" ht="24.75" spans="2:11">
-      <c r="B186" s="20">
+      <c r="J185" s="21">
+        <v>1</v>
+      </c>
+      <c r="K185" s="21"/>
+    </row>
+    <row r="186" spans="1:11" ht="24">
+      <c r="B186" s="19">
         <f>ROW(B186)-ROW($B$2)</f>
         <v>184</v>
       </c>
-      <c r="C186" s="21" t="s">
+      <c r="C186" s="20" t="s">
         <v>776</v>
       </c>
-      <c r="D186" s="22" t="s">
+      <c r="D186" s="21" t="s">
         <v>783</v>
       </c>
-      <c r="E186" s="22" t="s">
+      <c r="E186" s="21" t="s">
         <v>784</v>
       </c>
-      <c r="F186" s="22" t="s">
+      <c r="F186" s="21" t="s">
         <v>779</v>
       </c>
-      <c r="G186" s="22" t="s">
+      <c r="G186" s="21" t="s">
         <v>785</v>
       </c>
-      <c r="H186" s="22" t="s">
+      <c r="H186" s="21" t="s">
         <v>786</v>
       </c>
-      <c r="I186" s="22" t="s">
+      <c r="I186" s="21" t="s">
         <v>782</v>
       </c>
-      <c r="J186" s="22">
-        <v>1</v>
-      </c>
-      <c r="K186" s="22"/>
-    </row>
-    <row r="187" ht="15.75" spans="2:11">
-      <c r="B187" s="20">
+      <c r="J186" s="21">
+        <v>1</v>
+      </c>
+      <c r="K186" s="21"/>
+    </row>
+    <row r="187" spans="1:11">
+      <c r="B187" s="19">
         <f>ROW(B187)-ROW($B$2)</f>
         <v>185</v>
       </c>
-      <c r="C187" s="21" t="s">
+      <c r="C187" s="20" t="s">
         <v>776</v>
       </c>
-      <c r="D187" s="22" t="s">
+      <c r="D187" s="21" t="s">
         <v>787</v>
       </c>
-      <c r="E187" s="22" t="s">
+      <c r="E187" s="21" t="s">
         <v>788</v>
       </c>
-      <c r="F187" s="22" t="s">
+      <c r="F187" s="21" t="s">
         <v>779</v>
       </c>
-      <c r="G187" s="22" t="s">
+      <c r="G187" s="21" t="s">
         <v>789</v>
       </c>
-      <c r="H187" s="22" t="s">
+      <c r="H187" s="21" t="s">
         <v>786</v>
       </c>
-      <c r="I187" s="22" t="s">
+      <c r="I187" s="21" t="s">
         <v>782</v>
       </c>
-      <c r="J187" s="22">
+      <c r="J187" s="21">
         <v>35</v>
       </c>
-      <c r="K187" s="22"/>
+      <c r="K187" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#4 Mating connector receptacle and pin part# updated in eSpark and Client BOM
</commit_message>
<xml_diff>
--- a/Design-Files/MVP-Dash-v1.0/BOM/Client_BOM.xlsx
+++ b/Design-Files/MVP-Dash-v1.0/BOM/Client_BOM.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27726"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\alastair-baronessalpha\Design-Files\MVP-Dash-v1.0\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\eSpark-Consultants\alastair-baronessalpha\Design-Files\MVP-Dash-v1.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3F46FF7-86C0-41A8-8161-091A7B50C00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11850"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,8 +24,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -2386,28 +2385,28 @@
     <t xml:space="preserve">Mating Connector </t>
   </si>
   <si>
-    <t>3 35P 4mm - Automobile Connectors ROHS</t>
-  </si>
-  <si>
-    <t>K776280H-35-PTW</t>
-  </si>
-  <si>
-    <t>XKB Connection</t>
-  </si>
-  <si>
     <t>Mating pin Terminal</t>
   </si>
   <si>
-    <t>Automobile Connectors ROHS</t>
-  </si>
-  <si>
-    <t>K776280T-PSN</t>
+    <t>77138-101LF</t>
+  </si>
+  <si>
+    <t>Amphenol ICC</t>
+  </si>
+  <si>
+    <t>Rectangular Connector Pin</t>
+  </si>
+  <si>
+    <t>Rectangular Connector Housings Receptacle</t>
+  </si>
+  <si>
+    <t>90311-026LF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="14">
     <font>
       <sz val="11"/>
@@ -2686,9 +2685,6 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2697,6 +2693,9 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2978,7 +2977,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K187"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
@@ -3005,9 +3004,9 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="2"/>
@@ -5008,26 +5007,26 @@
         <f>ROW(B65)-ROW($B$2)</f>
         <v>63</v>
       </c>
-      <c r="C65" s="23" t="s">
+      <c r="C65" s="22" t="s">
         <v>274</v>
       </c>
-      <c r="D65" s="24" t="s">
+      <c r="D65" s="23" t="s">
         <v>275</v>
       </c>
-      <c r="E65" s="25" t="s">
+      <c r="E65" s="24" t="s">
         <v>276</v>
       </c>
-      <c r="F65" s="24" t="s">
+      <c r="F65" s="23" t="s">
         <v>277</v>
       </c>
-      <c r="G65" s="25" t="s">
+      <c r="G65" s="24" t="s">
         <v>278</v>
       </c>
-      <c r="H65" s="24"/>
-      <c r="I65" s="25" t="s">
+      <c r="H65" s="23"/>
+      <c r="I65" s="24" t="s">
         <v>278</v>
       </c>
-      <c r="J65" s="24">
+      <c r="J65" s="23">
         <v>1</v>
       </c>
       <c r="K65" s="16" t="s">
@@ -8850,16 +8849,16 @@
       <c r="D186" s="21" t="s">
         <v>783</v>
       </c>
-      <c r="E186" s="21" t="s">
-        <v>784</v>
+      <c r="E186" s="9" t="s">
+        <v>788</v>
       </c>
       <c r="F186" s="21" t="s">
         <v>779</v>
       </c>
-      <c r="G186" s="21" t="s">
-        <v>785</v>
-      </c>
-      <c r="H186" s="21" t="s">
+      <c r="G186" s="9" t="s">
+        <v>789</v>
+      </c>
+      <c r="H186" s="9" t="s">
         <v>786</v>
       </c>
       <c r="I186" s="21" t="s">
@@ -8879,25 +8878,25 @@
         <v>776</v>
       </c>
       <c r="D187" s="21" t="s">
+        <v>784</v>
+      </c>
+      <c r="E187" s="9" t="s">
         <v>787</v>
-      </c>
-      <c r="E187" s="21" t="s">
-        <v>788</v>
       </c>
       <c r="F187" s="21" t="s">
         <v>779</v>
       </c>
-      <c r="G187" s="21" t="s">
-        <v>789</v>
-      </c>
-      <c r="H187" s="21" t="s">
+      <c r="G187" s="9" t="s">
+        <v>785</v>
+      </c>
+      <c r="H187" s="9" t="s">
         <v>786</v>
       </c>
       <c r="I187" s="21" t="s">
         <v>782</v>
       </c>
       <c r="J187" s="21">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="K187" s="21"/>
     </row>

</xml_diff>